<commit_message>
Remove `AwaitingGameData` state and related files, introduce `UniversalUnit` and update unit handling with position tracking and enhanced protobuf definitions.
</commit_message>
<xml_diff>
--- a/Shared/Faction Data.xlsx
+++ b/Shared/Faction Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\worlds-collide-tbs\Shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4356FECB-36CA-447E-AC2F-8772E65B5274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3962EA-EF34-4E27-8810-EF58B8009111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -630,8 +630,9 @@
   <dimension ref="A3:K46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Remove `DefaultMovement` implementation, refactor unit-to-army data structures and counts, and extend protobuf definitions with new message types and fields.
</commit_message>
<xml_diff>
--- a/Shared/Faction Data.xlsx
+++ b/Shared/Faction Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\worlds-collide-tbs\Shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3962EA-EF34-4E27-8810-EF58B8009111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2D3882-3394-4EAC-A51A-59DC4C1B97AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="20760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="34">
   <si>
     <t>Description</t>
   </si>
@@ -121,6 +121,15 @@
   </si>
   <si>
     <t>Slow</t>
+  </si>
+  <si>
+    <t>Default 1</t>
+  </si>
+  <si>
+    <t>Default 2</t>
+  </si>
+  <si>
+    <t>Plague Spreaders 1</t>
   </si>
 </sst>
 </file>
@@ -1333,7 +1342,7 @@
         <v>17</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>15</v>
@@ -1359,7 +1368,7 @@
         <v>20</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1379,7 +1388,7 @@
         <v>30</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -1500,7 +1509,7 @@
         <v>20</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Sync movement between clients
</commit_message>
<xml_diff>
--- a/Shared/Faction Data.xlsx
+++ b/Shared/Faction Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\worlds-collide-tbs\Shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2D3882-3394-4EAC-A51A-59DC4C1B97AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E204F6A1-4859-4B4B-9DF0-52F355E37A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="20760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="35">
   <si>
     <t>Description</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>Plague Spreaders 1</t>
+  </si>
+  <si>
+    <t>Support</t>
   </si>
 </sst>
 </file>
@@ -591,6 +594,9 @@
       <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I4" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1302,6 +1308,9 @@
       </c>
       <c r="H4" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
@@ -1470,6 +1479,9 @@
       <c r="H4" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="I4" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="K4" s="1" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Combat DSL for server
</commit_message>
<xml_diff>
--- a/Shared/Faction Data.xlsx
+++ b/Shared/Faction Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\worlds-collide-tbs\Shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41642EA-FE9D-45D9-9DCA-CCFFE21BD980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85AF83AB-5767-4DAF-82FF-AF0286360B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="35">
   <si>
     <t>Description</t>
   </si>
@@ -99,12 +99,6 @@
     <t>We're The Rats!</t>
   </si>
   <si>
-    <t>Attack Name</t>
-  </si>
-  <si>
-    <t>Damage</t>
-  </si>
-  <si>
     <t>AP Cost</t>
   </si>
   <si>
@@ -129,10 +123,16 @@
     <t>Plague Spreaders 1</t>
   </si>
   <si>
-    <t>Support</t>
-  </si>
-  <si>
     <t>Skills</t>
+  </si>
+  <si>
+    <t>CombatString</t>
+  </si>
+  <si>
+    <t>Skill Name</t>
+  </si>
+  <si>
+    <t>Universal</t>
   </si>
 </sst>
 </file>
@@ -541,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:S20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -552,16 +552,16 @@
     <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="2.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="2.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="2.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -569,12 +569,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
@@ -594,43 +594,40 @@
       <c r="H4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>33</v>
+      <c r="J4" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="M4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="R4" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="T4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="17" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="18" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="19" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -642,46 +639,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04AD92E6-845E-499F-BA5C-893249301DDF}">
-  <dimension ref="A3:K46"/>
+  <dimension ref="A3:L46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
-      <c r="I3" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="K3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -690,17 +691,18 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="2"/>
+      <c r="J4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2">
         <v>1</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -712,8 +714,9 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -725,8 +728,9 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -738,8 +742,9 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -751,8 +756,9 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -764,8 +770,9 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -777,8 +784,9 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -790,8 +798,9 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -803,8 +812,9 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -816,8 +826,9 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -829,8 +840,9 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -842,8 +854,9 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -855,8 +868,9 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -868,8 +882,9 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -881,8 +896,9 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -894,8 +910,9 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -907,8 +924,9 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -920,8 +938,9 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L21" s="2"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -933,8 +952,9 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -946,8 +966,9 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L23" s="2"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -959,8 +980,9 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L24" s="2"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -972,8 +994,9 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L25" s="2"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -985,8 +1008,9 @@
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L26" s="2"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -998,8 +1022,9 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L27" s="2"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1011,8 +1036,9 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L28" s="2"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1024,8 +1050,9 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L29" s="2"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1037,8 +1064,9 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1050,8 +1078,9 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1063,8 +1092,9 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L32" s="2"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1076,8 +1106,9 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L33" s="2"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1089,8 +1120,9 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L34" s="2"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1102,8 +1134,9 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L35" s="2"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -1115,8 +1148,9 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L36" s="2"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1128,8 +1162,9 @@
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L37" s="2"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -1141,8 +1176,9 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L38" s="2"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1154,8 +1190,9 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L39" s="2"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1167,8 +1204,9 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L40" s="2"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -1180,8 +1218,9 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L41" s="2"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -1193,8 +1232,9 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L42" s="2"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -1206,8 +1246,9 @@
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L43" s="2"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -1219,8 +1260,9 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L44" s="2"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1232,8 +1274,9 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L45" s="2"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1245,6 +1288,7 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
+      <c r="L46" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1289,7 +1333,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
@@ -1308,9 +1352,6 @@
       </c>
       <c r="H4" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>10</v>
@@ -1351,7 +1392,7 @@
         <v>16</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>14</v>
@@ -1377,12 +1418,12 @@
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>15</v>
@@ -1394,10 +1435,10 @@
         <v>5</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -1459,7 +1500,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
@@ -1478,9 +1519,6 @@
       </c>
       <c r="H4" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>10</v>
@@ -1521,7 +1559,7 @@
         <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
pulling data from the DB and getting it to the client
</commit_message>
<xml_diff>
--- a/Shared/Faction Data.xlsx
+++ b/Shared/Faction Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\worlds-collide-tbs\Shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85AF83AB-5767-4DAF-82FF-AF0286360B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CE1CCD-8201-4778-9E7C-9D15A5B8FB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-29490" yWindow="2940" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="40">
   <si>
     <t>Description</t>
   </si>
@@ -133,6 +133,21 @@
   </si>
   <si>
     <t>Universal</t>
+  </si>
+  <si>
+    <t>Basic Attack</t>
+  </si>
+  <si>
+    <t>D(2)</t>
+  </si>
+  <si>
+    <t>Basic Strike</t>
+  </si>
+  <si>
+    <t>Attack</t>
+  </si>
+  <si>
+    <t>Cooldown</t>
   </si>
 </sst>
 </file>
@@ -639,18 +654,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04AD92E6-845E-499F-BA5C-893249301DDF}">
-  <dimension ref="A3:L46"/>
+  <dimension ref="A3:M46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
@@ -669,40 +685,62 @@
       <c r="F3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>39</v>
+      </c>
       <c r="I3" s="1"/>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="1"/>
+      <c r="K3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
       <c r="I4" s="2"/>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="2"/>
+      <c r="K4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K4" s="2">
+      <c r="L4" s="2">
         <v>1</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -715,8 +753,9 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5" s="2"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -729,8 +768,9 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="2"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -743,8 +783,9 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7" s="2"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -757,8 +798,9 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" s="2"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -771,8 +813,9 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M9" s="2"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -785,8 +828,9 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M10" s="2"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -799,8 +843,9 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M11" s="2"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -813,8 +858,9 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M12" s="2"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -827,8 +873,9 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M13" s="2"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -841,8 +888,9 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M14" s="2"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -855,8 +903,9 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M15" s="2"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -869,8 +918,9 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M16" s="2"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -883,8 +933,9 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M17" s="2"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -897,8 +948,9 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M18" s="2"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -911,8 +963,9 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M19" s="2"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -925,8 +978,9 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M20" s="2"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -939,8 +993,9 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M21" s="2"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -953,8 +1008,9 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M22" s="2"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -967,8 +1023,9 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M23" s="2"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -981,8 +1038,9 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M24" s="2"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -995,8 +1053,9 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M25" s="2"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1009,8 +1068,9 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M26" s="2"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1023,8 +1083,9 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M27" s="2"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1037,8 +1098,9 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M28" s="2"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1051,8 +1113,9 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M29" s="2"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1065,8 +1128,9 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M30" s="2"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1079,8 +1143,9 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M31" s="2"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1093,8 +1158,9 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M32" s="2"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1107,8 +1173,9 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M33" s="2"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1121,8 +1188,9 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M34" s="2"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1135,8 +1203,9 @@
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M35" s="2"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -1149,8 +1218,9 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M36" s="2"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1163,8 +1233,9 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M37" s="2"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -1177,8 +1248,9 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M38" s="2"/>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1191,8 +1263,9 @@
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M39" s="2"/>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1205,8 +1278,9 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M40" s="2"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -1219,8 +1293,9 @@
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M41" s="2"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -1233,8 +1308,9 @@
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M42" s="2"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -1247,8 +1323,9 @@
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M43" s="2"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -1261,8 +1338,9 @@
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M44" s="2"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1275,8 +1353,9 @@
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M45" s="2"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1289,6 +1368,7 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
+      <c r="M46" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixing unexpected crashes, data formatting on input, to remove spaces from skill names
</commit_message>
<xml_diff>
--- a/Shared/Faction Data.xlsx
+++ b/Shared/Faction Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matt\Documents\worlds-collide-tbs\Shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CE1CCD-8201-4778-9E7C-9D15A5B8FB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973164CC-848C-40A5-A213-2171364F706B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29490" yWindow="2940" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32670" yWindow="3645" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="40">
   <si>
     <t>Description</t>
   </si>
@@ -1384,11 +1384,11 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="2.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -1458,6 +1458,9 @@
     <row r="5" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>15</v>

</xml_diff>